<commit_message>
PFC: fz_source option, FEM verify refinements, template with 58 parameters
- size_cicc_cable/scan_wp_designs: fz_source (0 external net force, 1 FZmax
  from emag per candidate, 2 max of both) as a sizing option
- fem_pfc_verify: squeeze-based vertical stress, signed hoop, field maxima
  from cell-averaged field, hoop equilibrium check
- input template and params regenerated (58 parameters), README updated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SgU5uhxNo2P8j9g7q4htYR
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/PFC/input/WP_PFC_input_template.xlsx
+++ b/MADE-2.0/matlab/PFC/input/WP_PFC_input_template.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1357,16 +1357,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Fatigue (FCGR)</t>
+          <t>Materials &amp; allowables</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>fcgr_mode</t>
+          <t>fz_source</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0 = off, 1 = compute plasma_cycles for every accepted design, 2 = size the jacket until plasma_cycles &gt;= plasma_cycles_min</t>
+          <t>Axial force in the ring stress: 0 = external scenario force (FZ_PF.xlsx or computed from the scenarios, legacy), 1 = FZmax computed per candidate by emag_field_forces (self-field squeeze at the mid-plane), 2 = the larger of the two</t>
         </is>
       </c>
     </row>
@@ -1387,20 +1387,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>plasma_cycles_min</t>
+          <t>fcgr_mode</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>k cycles</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Minimum fatigue life (thousands of plasma cycles) enforced when fcgr_mode = 2</t>
+          <t>0 = off, 1 = compute plasma_cycles for every accepted design, 2 = size the jacket until plasma_cycles &gt;= plasma_cycles_min</t>
         </is>
       </c>
     </row>
@@ -1412,20 +1412,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>fcgr_C0</t>
+          <t>plasma_cycles_min</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3.86e-11</v>
+        <v>30</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>m/cycle*(MPa*sqrt(m))^-m</t>
+          <t>k cycles</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Paris law constant (316LN: 3.86e-11; JK2LB: 1.75e-13)</t>
+          <t>Minimum fatigue life (thousands of plasma cycles) enforced when fcgr_mode = 2</t>
         </is>
       </c>
     </row>
@@ -1437,20 +1437,20 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>fcgr_m</t>
+          <t>fcgr_C0</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2.394</v>
+        <v>3.86e-11</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m/cycle*(MPa*sqrt(m))^-m</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Paris law exponent (316LN: 2.394; JK2LB: 3.7)</t>
+          <t>Paris law constant (316LN: 3.86e-11; JK2LB: 1.75e-13)</t>
         </is>
       </c>
     </row>
@@ -1462,11 +1462,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>fcgr_mw</t>
+          <t>fcgr_m</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.5</v>
+        <v>2.394</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Walker exponent</t>
+          <t>Paris law exponent (316LN: 2.394; JK2LB: 3.7)</t>
         </is>
       </c>
     </row>
@@ -1487,20 +1487,20 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>fcgr_residual_stress</t>
+          <t>fcgr_mw</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>200</v>
+        <v>0.5</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>MPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Residual stress in the jacket (sets the minimum of the stress cycle)</t>
+          <t>Walker exponent</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>fcgr_KIC</t>
+          <t>fcgr_residual_stress</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1520,12 +1520,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>MPa*sqrt(m)</t>
+          <t>MPa</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fracture toughness of the jacket steel</t>
+          <t>Residual stress in the jacket (sets the minimum of the stress cycle)</t>
         </is>
       </c>
     </row>
@@ -1537,20 +1537,20 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>fcgr_flaw_aspect</t>
+          <t>fcgr_KIC</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3</v>
+        <v>200</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MPa*sqrt(m)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Initial flaw aspect ratio c0/a0 (ITER standard: 3)</t>
+          <t>Fracture toughness of the jacket steel</t>
         </is>
       </c>
     </row>
@@ -1562,11 +1562,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>fcgr_flaw_type</t>
+          <t>fcgr_flaw_aspect</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>0 = embedded flaw, 1 = surface flaw</t>
+          <t>Initial flaw aspect ratio c0/a0 (ITER standard: 3)</t>
         </is>
       </c>
     </row>
@@ -1587,45 +1587,45 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>fcgr_flaw_area</t>
+          <t>fcgr_flaw_type</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2e-06</v>
+        <v>1</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>m^2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Initial flaw area (surface: 2e-6, embedded: 5e-6 in the legacy code)</t>
+          <t>0 = embedded flaw, 1 = surface flaw</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>FEM verification</t>
+          <t>Fatigue (FCGR)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>fem_mesh_r</t>
+          <t>fcgr_flaw_area</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
+        <v>2e-06</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m^2</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Finite elements per turn in the radial direction</t>
+          <t>Initial flaw area (surface: 2e-6, embedded: 5e-6 in the legacy code)</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>fem_mesh_z</t>
+          <t>fem_mesh_r</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Finite elements per turn in the axial direction</t>
+          <t>Finite elements per turn in the radial direction</t>
         </is>
       </c>
     </row>
@@ -1662,11 +1662,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>fem_subfil</t>
+          <t>fem_mesh_z</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Sub-filaments per side used to represent each turn's uniform current in the field model</t>
+          <t>Finite elements per turn in the axial direction</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>fem_bg_fil_r</t>
+          <t>fem_subfil</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Radial filaments used for each background coil (CS, other PF, plasma)</t>
+          <t>Sub-filaments per side used to represent each turn's uniform current in the field model</t>
         </is>
       </c>
     </row>
@@ -1712,11 +1712,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>fem_bg_fil_z</t>
+          <t>fem_bg_fil_r</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Axial filaments used for each background coil</t>
+          <t>Radial filaments used for each background coil (CS, other PF, plasma)</t>
         </is>
       </c>
     </row>
@@ -1737,11 +1737,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>fem_bc</t>
+          <t>fem_bg_fil_z</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Vertical support: 1 = inertia relief (net axial force spread over the volume), 2 = rigid support of the bottom face</t>
+          <t>Axial filaments used for each background coil</t>
         </is>
       </c>
     </row>
@@ -1762,11 +1762,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>fem_nu_wp</t>
+          <t>fem_bc</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1775,32 +1775,32 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Poisson ratio of the homogenized winding pack</t>
+          <t>Vertical support: 1 = inertia relief (net axial force spread over the volume), 2 = rigid support of the bottom face</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Geometric checks</t>
+          <t>FEM verification</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SC_w_min</t>
+          <t>fem_nu_wp</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.005</v>
+        <v>0.3</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Minimum superconductor cable width accepted</t>
+          <t>Poisson ratio of the homogenized winding pack</t>
         </is>
       </c>
     </row>
@@ -1812,20 +1812,20 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>r_cable_min</t>
+          <t>SC_w_min</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>0.005</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Minimum accepted conductor aspect ratio Cond_h/Cond_w</t>
+          <t>Minimum superconductor cable width accepted</t>
         </is>
       </c>
     </row>
@@ -1837,11 +1837,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>r_cable_max</t>
+          <t>r_cable_min</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Maximum accepted conductor aspect ratio Cond_h/Cond_w</t>
+          <t>Minimum accepted conductor aspect ratio Cond_h/Cond_w</t>
         </is>
       </c>
     </row>
@@ -1862,18 +1862,43 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>r_cable_max</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Maximum accepted conductor aspect ratio Cond_h/Cond_w</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Geometric checks</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>WP_radial_build_max</t>
         </is>
       </c>
-      <c r="C58" t="n">
+      <c r="C59" t="n">
         <v>1</v>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Maximum accepted total radial build (Re-Ri) of the coil</t>
         </is>

</xml_diff>

<commit_message>
PFC: system-based sizing option, vertical stress pi factor corrected by default
- system_sizing input option (default 0): background field of CS/PF/plasma and
  per-scenario current and axial force, worst-case envelope in the stress check
- ring_Fz_area_fix default 1: S_ver = FZ/(pi*(Re^2-Ri^2)); 0 keeps the legacy form
- template/params regenerated (59 parameters), README updated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SgU5uhxNo2P8j9g7q4htYR
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/PFC/input/WP_PFC_input_template.xlsx
+++ b/MADE-2.0/matlab/PFC/input/WP_PFC_input_template.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -700,32 +700,32 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Background field from other coils/plasma added to each grade's self field</t>
+          <t>Constant background field added to each grade's self field (used with system_sizing = 0)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Coil build</t>
+          <t>Design point</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>grins_w</t>
+          <t>system_sizing</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Radial ground insulation thickness</t>
+          <t>0 = each coil is sized on its own field and the axial force given (no scenario needed); 1 = system-based sizing: background field of CS, other PF and plasma in every scenario of the geometry file, coil current and axial force per scenario, worst-case envelope</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>grins_h</t>
+          <t>grins_w</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Axial ground insulation thickness</t>
+          <t>Radial ground insulation thickness</t>
         </is>
       </c>
     </row>
@@ -762,11 +762,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tins</t>
+          <t>grins_h</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -775,7 +775,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Turn insulation thickness</t>
+          <t>Axial ground insulation thickness</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ins_grades</t>
+          <t>tins</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -800,7 +800,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Insulation thickness between grades</t>
+          <t>Turn insulation thickness</t>
         </is>
       </c>
     </row>
@@ -812,11 +812,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>spacer</t>
+          <t>ins_grades</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -825,23 +825,23 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Axial spacer thickness between series modules</t>
+          <t>Insulation thickness between grades</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Numerical settings</t>
+          <t>Coil build</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>min_size_CICC</t>
+          <t>spacer</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Minimum CICC conductor size, bounds the turns-per-layer search</t>
+          <t>Axial spacer thickness between series modules</t>
         </is>
       </c>
     </row>
@@ -862,11 +862,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>max_size_CICC</t>
+          <t>min_size_CICC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Maximum CICC conductor size, bounds the turns-per-layer search</t>
+          <t>Minimum CICC conductor size, bounds the turns-per-layer search</t>
         </is>
       </c>
     </row>
@@ -887,20 +887,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Iop_min</t>
+          <t>max_size_CICC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>30000</v>
+        <v>0.06</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Minimum operating current scanned</t>
+          <t>Maximum CICC conductor size, bounds the turns-per-layer search</t>
         </is>
       </c>
     </row>
@@ -912,11 +912,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Iop_max</t>
+          <t>Iop_min</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Maximum operating current scanned</t>
+          <t>Minimum operating current scanned</t>
         </is>
       </c>
     </row>
@@ -937,11 +937,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Iop_step</t>
+          <t>Iop_max</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1000</v>
+        <v>60000</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Operating current scan step</t>
+          <t>Maximum operating current scanned</t>
         </is>
       </c>
     </row>
@@ -962,20 +962,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>min_B</t>
+          <t>Iop_step</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>1000</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Minimum self field accepted by the pre-filter (ESTIMATE_PEAK_FIELD)</t>
+          <t>Operating current scan step</t>
         </is>
       </c>
     </row>
@@ -987,11 +987,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>max_B</t>
+          <t>min_B</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Maximum self field accepted by the pre-filter (ESTIMATE_PEAK_FIELD)</t>
+          <t>Minimum self field accepted by the pre-filter (ESTIMATE_PEAK_FIELD)</t>
         </is>
       </c>
     </row>
@@ -1012,20 +1012,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MAt_tolerance</t>
+          <t>max_B</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.1</v>
+        <v>10</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>A candidate is kept only if its Ampere-turns fall within [MAt_target, MAt_tolerance*MAt_target]</t>
+          <t>Maximum self field accepted by the pre-filter (ESTIMATE_PEAK_FIELD)</t>
         </is>
       </c>
     </row>
@@ -1037,20 +1037,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JT_min</t>
+          <t>MAt_tolerance</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.001</v>
+        <v>1.1</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Minimum (starting) jacket thickness in the sizing loop</t>
+          <t>A candidate is kept only if its Ampere-turns fall within [MAt_target, MAt_tolerance*MAt_target]</t>
         </is>
       </c>
     </row>
@@ -1062,11 +1062,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JT_step</t>
+          <t>JT_min</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.0001</v>
+        <v>0.001</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Jacket thickness increment per sizing iteration</t>
+          <t>Minimum (starting) jacket thickness in the sizing loop</t>
         </is>
       </c>
     </row>
@@ -1087,20 +1087,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>max_sizing_iterations</t>
+          <t>JT_step</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>200000</v>
+        <v>0.0001</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Safety cap on the JT-growing sizing loop (new: the legacy driver had no cap)</t>
+          <t>Jacket thickness increment per sizing iteration</t>
         </is>
       </c>
     </row>
@@ -1112,45 +1112,45 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tau_discharge_fixed</t>
+          <t>max_sizing_iterations</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>10</v>
+        <v>200000</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fixed discharge time used for the hot-spot and voltage calculations (the legacy driver derives the required voltage from it, not the other way round)</t>
+          <t>Safety cap on the JT-growing sizing loop (new: the legacy driver had no cap)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Materials &amp; allowables</t>
+          <t>Numerical settings</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>S_hoop_allow</t>
+          <t>Tau_discharge_fixed</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>667000000</v>
+        <v>10</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>s</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Base jacket allowable stress (steel yield-derived)</t>
+          <t>Fixed discharge time used for the hot-spot and voltage calculations (the legacy driver derives the required voltage from it, not the other way round)</t>
         </is>
       </c>
     </row>
@@ -1162,20 +1162,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SF_hoop</t>
+          <t>S_hoop_allow</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1.3</v>
+        <v>667000000</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pa</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Safety factor on S_hoop_allow for the hoop-stress limit</t>
+          <t>Base jacket allowable stress (steel yield-derived)</t>
         </is>
       </c>
     </row>
@@ -1187,11 +1187,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tresca_factor</t>
+          <t>SF_hoop</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Multiplier on the hoop allowable for the Tresca-stress limit</t>
+          <t>Safety factor on S_hoop_allow for the hoop-stress limit</t>
         </is>
       </c>
     </row>
@@ -1212,20 +1212,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>E_jckt</t>
+          <t>Tresca_factor</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>205</v>
+        <v>1.5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Jacket (steel) Young's modulus, used by the ring stress model and the FEM homogenization</t>
+          <t>Multiplier on the hoop allowable for the Tresca-stress limit</t>
         </is>
       </c>
     </row>
@@ -1237,11 +1237,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>E_cbl_LTS</t>
+          <t>E_jckt</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.1</v>
+        <v>205</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Equivalent Young's modulus of an LTS cable (strand bundle, voids): carries almost no load</t>
+          <t>Jacket (steel) Young's modulus, used by the ring stress model and the FEM homogenization</t>
         </is>
       </c>
     </row>
@@ -1262,11 +1262,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>E_cbl_HTS</t>
+          <t>E_cbl_LTS</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>120</v>
+        <v>0.1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Equivalent Young's modulus of an HTS cable</t>
+          <t>Equivalent Young's modulus of an LTS cable (strand bundle, voids): carries almost no load</t>
         </is>
       </c>
     </row>
@@ -1287,11 +1287,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>E_ins</t>
+          <t>E_cbl_HTS</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Turn insulation Young's modulus</t>
+          <t>Equivalent Young's modulus of an HTS cable</t>
         </is>
       </c>
     </row>
@@ -1312,20 +1312,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ring_nu</t>
+          <t>E_ins</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.3333333</v>
+        <v>20</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Poisson ratio used by the thick-ring stress formula</t>
+          <t>Turn insulation Young's modulus</t>
         </is>
       </c>
     </row>
@@ -1337,11 +1337,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ring_Fz_area_fix</t>
+          <t>ring_nu</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>0.3333333</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>0 = legacy vertical stress FZ/(Re^2-Ri^2)*pi (kept as legacy default); 1 = annulus-area form FZ/(pi*(Re^2-Ri^2)). See manuale PFC, revisione modelli</t>
+          <t>Poisson ratio used by the thick-ring stress formula</t>
         </is>
       </c>
     </row>
@@ -1362,11 +1362,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>fz_source</t>
+          <t>ring_Fz_area_fix</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1375,23 +1375,23 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Axial force in the ring stress: 0 = external scenario force (FZ_PF.xlsx or computed from the scenarios, legacy), 1 = FZmax computed per candidate by emag_field_forces (self-field squeeze at the mid-plane), 2 = the larger of the two</t>
+          <t>1 = vertical stress FZ/(pi*(Re^2-Ri^2)) (annulus area, corrected); 0 = legacy FZ/(Re^2-Ri^2)*pi, which overestimates by pi^2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Fatigue (FCGR)</t>
+          <t>Materials &amp; allowables</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>fcgr_mode</t>
+          <t>fz_source</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>0 = off, 1 = compute plasma_cycles for every accepted design, 2 = size the jacket until plasma_cycles &gt;= plasma_cycles_min</t>
+          <t>Axial force in the ring stress: 0 = external scenario force (FZ_PF.xlsx or computed from the scenarios, legacy), 1 = FZmax computed per candidate by emag_field_forces (self-field squeeze at the mid-plane), 2 = the larger of the two</t>
         </is>
       </c>
     </row>
@@ -1412,20 +1412,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>plasma_cycles_min</t>
+          <t>fcgr_mode</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>k cycles</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Minimum fatigue life (thousands of plasma cycles) enforced when fcgr_mode = 2</t>
+          <t>0 = off, 1 = compute plasma_cycles for every accepted design, 2 = size the jacket until plasma_cycles &gt;= plasma_cycles_min</t>
         </is>
       </c>
     </row>
@@ -1437,20 +1437,20 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>fcgr_C0</t>
+          <t>plasma_cycles_min</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3.86e-11</v>
+        <v>30</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>m/cycle*(MPa*sqrt(m))^-m</t>
+          <t>k cycles</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Paris law constant (316LN: 3.86e-11; JK2LB: 1.75e-13)</t>
+          <t>Minimum fatigue life (thousands of plasma cycles) enforced when fcgr_mode = 2</t>
         </is>
       </c>
     </row>
@@ -1462,20 +1462,20 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>fcgr_m</t>
+          <t>fcgr_C0</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2.394</v>
+        <v>3.86e-11</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m/cycle*(MPa*sqrt(m))^-m</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Paris law exponent (316LN: 2.394; JK2LB: 3.7)</t>
+          <t>Paris law constant (316LN: 3.86e-11; JK2LB: 1.75e-13)</t>
         </is>
       </c>
     </row>
@@ -1487,11 +1487,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>fcgr_mw</t>
+          <t>fcgr_m</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.5</v>
+        <v>2.394</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Walker exponent</t>
+          <t>Paris law exponent (316LN: 2.394; JK2LB: 3.7)</t>
         </is>
       </c>
     </row>
@@ -1512,20 +1512,20 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>fcgr_residual_stress</t>
+          <t>fcgr_mw</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>200</v>
+        <v>0.5</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>MPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Residual stress in the jacket (sets the minimum of the stress cycle)</t>
+          <t>Walker exponent</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>fcgr_KIC</t>
+          <t>fcgr_residual_stress</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1545,12 +1545,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>MPa*sqrt(m)</t>
+          <t>MPa</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Fracture toughness of the jacket steel</t>
+          <t>Residual stress in the jacket (sets the minimum of the stress cycle)</t>
         </is>
       </c>
     </row>
@@ -1562,20 +1562,20 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>fcgr_flaw_aspect</t>
+          <t>fcgr_KIC</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>200</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MPa*sqrt(m)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Initial flaw aspect ratio c0/a0 (ITER standard: 3)</t>
+          <t>Fracture toughness of the jacket steel</t>
         </is>
       </c>
     </row>
@@ -1587,11 +1587,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>fcgr_flaw_type</t>
+          <t>fcgr_flaw_aspect</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0 = embedded flaw, 1 = surface flaw</t>
+          <t>Initial flaw aspect ratio c0/a0 (ITER standard: 3)</t>
         </is>
       </c>
     </row>
@@ -1612,45 +1612,45 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>fcgr_flaw_area</t>
+          <t>fcgr_flaw_type</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2e-06</v>
+        <v>1</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>m^2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Initial flaw area (surface: 2e-6, embedded: 5e-6 in the legacy code)</t>
+          <t>0 = embedded flaw, 1 = surface flaw</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>FEM verification</t>
+          <t>Fatigue (FCGR)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>fem_mesh_r</t>
+          <t>fcgr_flaw_area</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>2e-06</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m^2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Finite elements per turn in the radial direction</t>
+          <t>Initial flaw area (surface: 2e-6, embedded: 5e-6 in the legacy code)</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>fem_mesh_z</t>
+          <t>fem_mesh_r</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Finite elements per turn in the axial direction</t>
+          <t>Finite elements per turn in the radial direction</t>
         </is>
       </c>
     </row>
@@ -1687,11 +1687,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>fem_subfil</t>
+          <t>fem_mesh_z</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Sub-filaments per side used to represent each turn's uniform current in the field model</t>
+          <t>Finite elements per turn in the axial direction</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>fem_bg_fil_r</t>
+          <t>fem_subfil</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Radial filaments used for each background coil (CS, other PF, plasma)</t>
+          <t>Sub-filaments per side used to represent each turn's uniform current in the field model</t>
         </is>
       </c>
     </row>
@@ -1737,11 +1737,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>fem_bg_fil_z</t>
+          <t>fem_bg_fil_r</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Axial filaments used for each background coil</t>
+          <t>Radial filaments used for each background coil (CS, other PF, plasma)</t>
         </is>
       </c>
     </row>
@@ -1762,11 +1762,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>fem_bc</t>
+          <t>fem_bg_fil_z</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Vertical support: 1 = inertia relief (net axial force spread over the volume), 2 = rigid support of the bottom face</t>
+          <t>Axial filaments used for each background coil</t>
         </is>
       </c>
     </row>
@@ -1787,11 +1787,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>fem_nu_wp</t>
+          <t>fem_bc</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1800,32 +1800,32 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Poisson ratio of the homogenized winding pack</t>
+          <t>Vertical support: 1 = inertia relief (net axial force spread over the volume), 2 = rigid support of the bottom face</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Geometric checks</t>
+          <t>FEM verification</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SC_w_min</t>
+          <t>fem_nu_wp</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.005</v>
+        <v>0.3</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Minimum superconductor cable width accepted</t>
+          <t>Poisson ratio of the homogenized winding pack</t>
         </is>
       </c>
     </row>
@@ -1837,20 +1837,20 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>r_cable_min</t>
+          <t>SC_w_min</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>0.005</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Minimum accepted conductor aspect ratio Cond_h/Cond_w</t>
+          <t>Minimum superconductor cable width accepted</t>
         </is>
       </c>
     </row>
@@ -1862,11 +1862,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>r_cable_max</t>
+          <t>r_cable_min</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Maximum accepted conductor aspect ratio Cond_h/Cond_w</t>
+          <t>Minimum accepted conductor aspect ratio Cond_h/Cond_w</t>
         </is>
       </c>
     </row>
@@ -1887,18 +1887,43 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>r_cable_max</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Maximum accepted conductor aspect ratio Cond_h/Cond_w</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Geometric checks</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>WP_radial_build_max</t>
         </is>
       </c>
-      <c r="C59" t="n">
+      <c r="C60" t="n">
         <v>1</v>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Maximum accepted total radial build (Re-Ri) of the coil</t>
         </is>

</xml_diff>

<commit_message>
PFC: allinea ai fix del CS (Ic_sst33 B/T, forza assiale per candidato)
- size_conductor_cicc: Ic_sst33(B_local, T_dim, ...) nell'ordine corretto
- fz_source default 1: FZmax calcolato da emag per candidato (come nel CS)
- template, params di test e README aggiornati

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SgU5uhxNo2P8j9g7q4htYR
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/PFC/input/WP_PFC_input_template.xlsx
+++ b/MADE-2.0/matlab/PFC/input/WP_PFC_input_template.xlsx
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Axial force in the ring stress: 0 = external scenario force (FZ_PF.xlsx or computed from the scenarios, legacy), 1 = FZmax computed per candidate by emag_field_forces (self-field squeeze at the mid-plane), 2 = the larger of the two</t>
+          <t>Axial force in the ring stress: 1 = FZmax computed per candidate by emag_field_forces (self-field squeeze at the mid-plane, as in CS); 0 = external scenario force (FZ_PF.xlsx or computed from the scenarios, legacy); 2 = the larger of the two</t>
         </is>
       </c>
     </row>

</xml_diff>